<commit_message>
Added delay example usage
</commit_message>
<xml_diff>
--- a/examples/demo/simple_demo.xlsx
+++ b/examples/demo/simple_demo.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="tr0001" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="85">
   <si>
     <t xml:space="preserve">tr_uuid:</t>
   </si>
@@ -269,6 +269,9 @@
     <t xml:space="preserve">--headless</t>
   </si>
   <si>
+    <t xml:space="preserve">delay,5</t>
+  </si>
+  <si>
     <t xml:space="preserve">firefox</t>
   </si>
   <si>
@@ -276,6 +279,9 @@
   </si>
   <si>
     <t xml:space="preserve">explicit_wait,30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delayMax,1</t>
   </si>
 </sst>
 </file>
@@ -629,7 +635,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -652,10 +658,10 @@
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -710,7 +716,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -785,7 +791,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="2" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="40.71"/>
@@ -1007,7 +1013,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="2" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="28.57"/>
@@ -1290,7 +1296,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.86"/>
@@ -1362,8 +1368,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.42"/>
@@ -1420,6 +1426,11 @@
       </c>
       <c r="D4" s="1" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1438,8 +1449,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.86"/>
@@ -1459,7 +1470,7 @@
         <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1478,7 +1489,7 @@
         <v>72</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>74</v>
@@ -1492,7 +1503,12 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1512,7 +1528,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.86"/>
@@ -1532,7 +1548,7 @@
         <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1551,7 +1567,7 @@
         <v>72</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>74</v>
@@ -1563,7 +1579,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added delay, and variable delay (#240)
* Added delay, and variable delay

* Added delay example usage
</commit_message>
<xml_diff>
--- a/examples/demo/simple_demo.xlsx
+++ b/examples/demo/simple_demo.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="tr0001" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="85">
   <si>
     <t xml:space="preserve">tr_uuid:</t>
   </si>
@@ -269,6 +269,9 @@
     <t xml:space="preserve">--headless</t>
   </si>
   <si>
+    <t xml:space="preserve">delay,5</t>
+  </si>
+  <si>
     <t xml:space="preserve">firefox</t>
   </si>
   <si>
@@ -276,6 +279,9 @@
   </si>
   <si>
     <t xml:space="preserve">explicit_wait,30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delayMax,1</t>
   </si>
 </sst>
 </file>
@@ -629,7 +635,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -652,10 +658,10 @@
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -710,7 +716,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -785,7 +791,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="2" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="40.71"/>
@@ -1007,7 +1013,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="2" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="28.57"/>
@@ -1290,7 +1296,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.86"/>
@@ -1362,8 +1368,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.42"/>
@@ -1420,6 +1426,11 @@
       </c>
       <c r="D4" s="1" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1438,8 +1449,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.86"/>
@@ -1459,7 +1470,7 @@
         <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1478,7 +1489,7 @@
         <v>72</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>74</v>
@@ -1492,7 +1503,12 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="1" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1512,7 +1528,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.86"/>
@@ -1532,7 +1548,7 @@
         <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1551,7 +1567,7 @@
         <v>72</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>74</v>
@@ -1563,7 +1579,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>